<commit_message>
BLAST Premier 2026 Seoul Playoffs
</commit_message>
<xml_diff>
--- a/file/finances_updated.xlsx
+++ b/file/finances_updated.xlsx
@@ -1,563 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joao.abraga\Downloads\ck-tools-main\file\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DA600F-7BFB-4638-83C0-69A794EEC67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="1815" yWindow="2670" windowWidth="18030" windowHeight="10875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
     <sheet name="Finances" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="177">
-  <si>
-    <t>TeamName</t>
-  </si>
-  <si>
-    <t>Tier</t>
-  </si>
-  <si>
-    <t>CurrentBank</t>
-  </si>
-  <si>
-    <t>Coach</t>
-  </si>
-  <si>
-    <t>Analyst</t>
-  </si>
-  <si>
-    <t>HeathTeam</t>
-  </si>
-  <si>
-    <t>PhysicalTeam</t>
-  </si>
-  <si>
-    <t>Maintenance</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>00 Nation</t>
-  </si>
-  <si>
-    <t>Tier 3</t>
-  </si>
-  <si>
-    <t>100 Thieves</t>
-  </si>
-  <si>
-    <t>3DMAX</t>
-  </si>
-  <si>
-    <t>9Pandas</t>
-  </si>
-  <si>
-    <t>9z</t>
-  </si>
-  <si>
-    <t>ad hoc</t>
-  </si>
-  <si>
-    <t>Aether</t>
-  </si>
-  <si>
-    <t>Alliance</t>
-  </si>
-  <si>
-    <t>AMKAL</t>
-  </si>
-  <si>
-    <t>Aravt</t>
-  </si>
-  <si>
-    <t>ARCRED</t>
-  </si>
-  <si>
-    <t>Astana Dragons</t>
-  </si>
-  <si>
-    <t>Astralis</t>
-  </si>
-  <si>
-    <t>Astralis Talent</t>
-  </si>
-  <si>
-    <t>ATOX</t>
-  </si>
-  <si>
-    <t>Aurora</t>
-  </si>
-  <si>
-    <t>Avangar</t>
-  </si>
-  <si>
-    <t>B8</t>
-  </si>
-  <si>
-    <t>Bad News Eagles</t>
-  </si>
-  <si>
-    <t>BC.Game</t>
-  </si>
-  <si>
-    <t>BESTIA</t>
-  </si>
-  <si>
-    <t>BIG</t>
-  </si>
-  <si>
-    <t>BIG Academy</t>
-  </si>
-  <si>
-    <t>Bounty Hunters</t>
-  </si>
-  <si>
-    <t>Bravado</t>
-  </si>
-  <si>
-    <t>Carnival</t>
-  </si>
-  <si>
-    <t>Case</t>
-  </si>
-  <si>
-    <t>CatEvil</t>
-  </si>
-  <si>
-    <t>Chinggis Warriors</t>
-  </si>
-  <si>
-    <t>Cloud9</t>
-  </si>
-  <si>
-    <t>Complexity</t>
-  </si>
-  <si>
-    <t>Copenhagen Flames</t>
-  </si>
-  <si>
-    <t>Copenhagen Wolves</t>
-  </si>
-  <si>
-    <t>Counter Logic</t>
-  </si>
-  <si>
-    <t>devils.one</t>
-  </si>
-  <si>
-    <t>Dignitas</t>
-  </si>
-  <si>
-    <t>ECSTATIC</t>
-  </si>
-  <si>
-    <t>Elevate</t>
-  </si>
-  <si>
-    <t>ENCE</t>
-  </si>
-  <si>
-    <t>ENCE Academy</t>
-  </si>
-  <si>
-    <t>Enemy</t>
-  </si>
-  <si>
-    <t>Entropiq</t>
-  </si>
-  <si>
-    <t>Envy</t>
-  </si>
-  <si>
-    <t>ESC</t>
-  </si>
-  <si>
-    <t>Eternal Fire</t>
-  </si>
-  <si>
-    <t>Evil Geniuses</t>
-  </si>
-  <si>
-    <t>Falcons</t>
-  </si>
-  <si>
-    <t>FaZe</t>
-  </si>
-  <si>
-    <t>Flash</t>
-  </si>
-  <si>
-    <t>FLuffy Gangsters</t>
-  </si>
-  <si>
-    <t>FlyQuest</t>
-  </si>
-  <si>
-    <t>FlyQuest RED</t>
-  </si>
-  <si>
-    <t>Fnatic</t>
-  </si>
-  <si>
-    <t>FORZE</t>
-  </si>
-  <si>
-    <t>FURIA</t>
-  </si>
-  <si>
-    <t>G2</t>
-  </si>
-  <si>
-    <t>Galorys</t>
-  </si>
-  <si>
-    <t>Gambit</t>
-  </si>
-  <si>
-    <t>GamerLegion</t>
-  </si>
-  <si>
-    <t>GATERON</t>
-  </si>
-  <si>
-    <t>GhoulsW</t>
-  </si>
-  <si>
-    <t>Gods Reign</t>
-  </si>
-  <si>
-    <t>GODSENT</t>
-  </si>
-  <si>
-    <t>HAVU</t>
-  </si>
-  <si>
-    <t>Heroic</t>
-  </si>
-  <si>
-    <t>Heroic Academy</t>
-  </si>
-  <si>
-    <t>Hesta</t>
-  </si>
-  <si>
-    <t>Homyno</t>
-  </si>
-  <si>
-    <t>hoorai</t>
-  </si>
-  <si>
-    <t>iBUYPOWER</t>
-  </si>
-  <si>
-    <t>IHC</t>
-  </si>
-  <si>
-    <t>Iluminar</t>
-  </si>
-  <si>
-    <t>Tier 2</t>
-  </si>
-  <si>
-    <t>Immortals</t>
-  </si>
-  <si>
-    <t>Imperial</t>
-  </si>
-  <si>
-    <t>inSanitY</t>
-  </si>
-  <si>
-    <t>Into the Beach</t>
-  </si>
-  <si>
-    <t>Kappa Bar</t>
-  </si>
-  <si>
-    <t>kONO</t>
-  </si>
-  <si>
-    <t>KRU</t>
-  </si>
-  <si>
-    <t>LDLC</t>
-  </si>
-  <si>
-    <t>Legacy</t>
-  </si>
-  <si>
-    <t>LGB</t>
-  </si>
-  <si>
-    <t>Limitless</t>
-  </si>
-  <si>
-    <t>Liquid</t>
-  </si>
-  <si>
-    <t>Luminosity</t>
-  </si>
-  <si>
-    <t>Lynn Vision</t>
-  </si>
-  <si>
-    <t>M80</t>
-  </si>
-  <si>
-    <t>MAD Lions</t>
-  </si>
-  <si>
-    <t>MANA</t>
-  </si>
-  <si>
-    <t>MenaceGG</t>
-  </si>
-  <si>
-    <t>MIBR</t>
-  </si>
-  <si>
-    <t>MIBR Academy</t>
-  </si>
-  <si>
-    <t>Misfits</t>
-  </si>
-  <si>
-    <t>mousesports</t>
-  </si>
-  <si>
-    <t>MOUZ</t>
-  </si>
-  <si>
-    <t>MOUZ NXT</t>
-  </si>
-  <si>
-    <t>Movistar KOI</t>
-  </si>
-  <si>
-    <t>Mythic</t>
-  </si>
-  <si>
-    <t>Natus Vincere</t>
-  </si>
-  <si>
-    <t>NAVI Junior</t>
-  </si>
-  <si>
-    <t>Nemiga</t>
-  </si>
-  <si>
-    <t>Nexus</t>
-  </si>
-  <si>
-    <t>Ninjas in Pyjamas</t>
-  </si>
-  <si>
-    <t>NIP Impact</t>
-  </si>
-  <si>
-    <t>NomadS</t>
-  </si>
-  <si>
-    <t>Nordix</t>
-  </si>
-  <si>
-    <t>NOVAQ</t>
-  </si>
-  <si>
-    <t>ODDIK</t>
-  </si>
-  <si>
-    <t>OG</t>
-  </si>
-  <si>
-    <t>Onyx Ravens</t>
-  </si>
-  <si>
-    <t>Orbit</t>
-  </si>
-  <si>
-    <t>Outsiders</t>
-  </si>
-  <si>
-    <t>paiN</t>
-  </si>
-  <si>
-    <t>paiN Academy</t>
-  </si>
-  <si>
-    <t>PARIVISION</t>
-  </si>
-  <si>
-    <t>Passion UA</t>
-  </si>
-  <si>
-    <t>Permitta</t>
-  </si>
-  <si>
-    <t>Qiang</t>
-  </si>
-  <si>
-    <t>QMISTRY</t>
-  </si>
-  <si>
-    <t>Quantum Bellator Fire</t>
-  </si>
-  <si>
-    <t>Reason</t>
-  </si>
-  <si>
-    <t>Rebels</t>
-  </si>
-  <si>
-    <t>RED Canids</t>
-  </si>
-  <si>
-    <t>Red Viperz</t>
-  </si>
-  <si>
-    <t>Rogue</t>
-  </si>
-  <si>
-    <t>Sangal</t>
-  </si>
-  <si>
-    <t>SAW</t>
-  </si>
-  <si>
-    <t>Sharks</t>
-  </si>
-  <si>
-    <t>Shika</t>
-  </si>
-  <si>
-    <t>ShindeN</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>Skinvault</t>
-  </si>
-  <si>
-    <t>SKYFURY</t>
-  </si>
-  <si>
-    <t>Space Soldiers</t>
-  </si>
-  <si>
-    <t>Spirit</t>
-  </si>
-  <si>
-    <t>Spirit Academy</t>
-  </si>
-  <si>
-    <t>Sprout</t>
-  </si>
-  <si>
-    <t>Take Flyte</t>
-  </si>
-  <si>
-    <t>TALON</t>
-  </si>
-  <si>
-    <t>Kinguin</t>
-  </si>
-  <si>
-    <t>Solid</t>
-  </si>
-  <si>
-    <t>The Dice</t>
-  </si>
-  <si>
-    <t>The Huns</t>
-  </si>
-  <si>
-    <t>The MongolZ</t>
-  </si>
-  <si>
-    <t>Titan</t>
-  </si>
-  <si>
-    <t>Tricked</t>
-  </si>
-  <si>
-    <t>True Rippers</t>
-  </si>
-  <si>
-    <t>Tsunami</t>
-  </si>
-  <si>
-    <t>TYLOO</t>
-  </si>
-  <si>
-    <t>Underground</t>
-  </si>
-  <si>
-    <t>Vantage</t>
-  </si>
-  <si>
-    <t>Venom</t>
-  </si>
-  <si>
-    <t>Verdant</t>
-  </si>
-  <si>
-    <t>VeryGames</t>
-  </si>
-  <si>
-    <t>Vexed</t>
-  </si>
-  <si>
-    <t>Victores Sumus</t>
-  </si>
-  <si>
-    <t>Virtus.pro</t>
-  </si>
-  <si>
-    <t>Vitality</t>
-  </si>
-  <si>
-    <t>Vox Eminor</t>
-  </si>
-  <si>
-    <t>VP.Prodigy</t>
-  </si>
-  <si>
-    <t>Wildcard</t>
-  </si>
-  <si>
-    <t>Wildcard Academy</t>
-  </si>
-  <si>
-    <t>Wings Up</t>
-  </si>
-  <si>
-    <t>Wizards</t>
-  </si>
-  <si>
-    <t>Lux Tenebris</t>
-  </si>
-  <si>
-    <t>Core</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -587,21 +65,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -926,45 +396,44 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I167"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TeamName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tier</v>
+      </c>
+      <c r="C1" t="str">
+        <v>CurrentBank</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Coach</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Analyst</v>
+      </c>
+      <c r="F1" t="str">
+        <v>HeathTeam</v>
+      </c>
+      <c r="G1" t="str">
+        <v>PhysicalTeam</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Maintenance</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Marketing</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>00 Nation</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C2">
         <v>28500</v>
@@ -988,12 +457,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>100 Thieves</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C3">
         <v>28500</v>
@@ -1017,12 +486,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>3DMAX</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C4">
         <v>28500</v>
@@ -1046,12 +515,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>9Pandas</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C5">
         <v>28500</v>
@@ -1075,12 +544,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>9z</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C6">
         <v>28500</v>
@@ -1104,12 +573,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ad hoc</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C7">
         <v>28500</v>
@@ -1133,12 +602,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Aether</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C8">
         <v>28500</v>
@@ -1162,12 +631,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>10</v>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Alliance</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C9">
         <v>28500</v>
@@ -1191,12 +660,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>AMKAL</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C10">
         <v>29700</v>
@@ -1220,12 +689,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>10</v>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Aravt</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C11">
         <v>28500</v>
@@ -1249,12 +718,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>10</v>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ARCRED</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C12">
         <v>28500</v>
@@ -1278,12 +747,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" t="s">
-        <v>10</v>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Astana Dragons</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C13">
         <v>29400</v>
@@ -1307,15 +776,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" t="s">
-        <v>10</v>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Astralis</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C14">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D14">
         <v>500</v>
@@ -1336,12 +805,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" t="s">
-        <v>10</v>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Astralis Talent</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C15">
         <v>28500</v>
@@ -1365,12 +834,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" t="s">
-        <v>10</v>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>ATOX</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C16">
         <v>28500</v>
@@ -1394,12 +863,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" t="s">
-        <v>10</v>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Aurora</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C17">
         <v>28500</v>
@@ -1423,12 +892,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" t="s">
-        <v>10</v>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Avangar</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C18">
         <v>28500</v>
@@ -1452,12 +921,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" t="s">
-        <v>10</v>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>B8</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C19">
         <v>28500</v>
@@ -1481,12 +950,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" t="s">
-        <v>10</v>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Bad News Eagles</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C20">
         <v>28500</v>
@@ -1510,15 +979,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B21" t="s">
-        <v>10</v>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>BC.Game</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C21">
-        <v>28500</v>
+        <v>29400</v>
       </c>
       <c r="D21">
         <v>500</v>
@@ -1539,12 +1008,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" t="s">
-        <v>10</v>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>BESTIA</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C22">
         <v>42100</v>
@@ -1568,12 +1037,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" t="s">
-        <v>10</v>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>BIG</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C23">
         <v>28500</v>
@@ -1597,12 +1066,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" t="s">
-        <v>10</v>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>BIG Academy</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C24">
         <v>28920</v>
@@ -1626,12 +1095,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" t="s">
-        <v>10</v>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Bounty Hunters</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C25">
         <v>42100</v>
@@ -1655,12 +1124,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" t="s">
-        <v>10</v>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Bravado</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C26">
         <v>28500</v>
@@ -1684,12 +1153,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>35</v>
-      </c>
-      <c r="B27" t="s">
-        <v>10</v>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Carnival</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C27">
         <v>28500</v>
@@ -1713,12 +1182,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B28" t="s">
-        <v>10</v>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Case</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C28">
         <v>28500</v>
@@ -1742,12 +1211,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" t="s">
-        <v>10</v>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>CatEvil</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C29">
         <v>28500</v>
@@ -1771,12 +1240,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>38</v>
-      </c>
-      <c r="B30" t="s">
-        <v>10</v>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Chinggis Warriors</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C30">
         <v>28500</v>
@@ -1800,12 +1269,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" t="s">
-        <v>10</v>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Cloud9</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C31">
         <v>44900</v>
@@ -1829,12 +1298,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>40</v>
-      </c>
-      <c r="B32" t="s">
-        <v>10</v>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Complexity</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C32">
         <v>28500</v>
@@ -1858,12 +1327,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" t="s">
-        <v>10</v>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Copenhagen Flames</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C33">
         <v>78700</v>
@@ -1887,12 +1356,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>42</v>
-      </c>
-      <c r="B34" t="s">
-        <v>10</v>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Copenhagen Wolves</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C34">
         <v>28920</v>
@@ -1916,12 +1385,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>43</v>
-      </c>
-      <c r="B35" t="s">
-        <v>10</v>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Counter Logic</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C35">
         <v>28500</v>
@@ -1945,12 +1414,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>44</v>
-      </c>
-      <c r="B36" t="s">
-        <v>10</v>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>devils.one</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C36">
         <v>28500</v>
@@ -1974,12 +1443,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>45</v>
-      </c>
-      <c r="B37" t="s">
-        <v>10</v>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Dignitas</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C37">
         <v>28500</v>
@@ -2003,12 +1472,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>46</v>
-      </c>
-      <c r="B38" t="s">
-        <v>10</v>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>ECSTATIC</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C38">
         <v>28500</v>
@@ -2032,12 +1501,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>47</v>
-      </c>
-      <c r="B39" t="s">
-        <v>10</v>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Elevate</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C39">
         <v>54500</v>
@@ -2061,12 +1530,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>48</v>
-      </c>
-      <c r="B40" t="s">
-        <v>10</v>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>ENCE</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C40">
         <v>28500</v>
@@ -2090,12 +1559,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>49</v>
-      </c>
-      <c r="B41" t="s">
-        <v>10</v>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>ENCE Academy</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C41">
         <v>28920</v>
@@ -2119,15 +1588,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>50</v>
-      </c>
-      <c r="B42" t="s">
-        <v>10</v>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Enemy</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C42">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D42">
         <v>500</v>
@@ -2148,12 +1617,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>51</v>
-      </c>
-      <c r="B43" t="s">
-        <v>10</v>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Entropiq</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C43">
         <v>29400</v>
@@ -2177,15 +1646,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>52</v>
-      </c>
-      <c r="B44" t="s">
-        <v>10</v>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Envy</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C44">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D44">
         <v>500</v>
@@ -2206,12 +1675,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B45" t="s">
-        <v>10</v>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>ESC</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C45">
         <v>28500</v>
@@ -2235,12 +1704,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>54</v>
-      </c>
-      <c r="B46" t="s">
-        <v>10</v>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Eternal Fire</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C46">
         <v>54500</v>
@@ -2264,12 +1733,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>55</v>
-      </c>
-      <c r="B47" t="s">
-        <v>10</v>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Evil Geniuses</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C47">
         <v>28500</v>
@@ -2293,15 +1762,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>56</v>
-      </c>
-      <c r="B48" t="s">
-        <v>10</v>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Falcons</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C48">
-        <v>138785.71428571429</v>
+        <v>138785.7142857143</v>
       </c>
       <c r="D48">
         <v>500</v>
@@ -2322,12 +1791,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>57</v>
-      </c>
-      <c r="B49" t="s">
-        <v>10</v>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>FaZe</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C49">
         <v>28500</v>
@@ -2351,12 +1820,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>58</v>
-      </c>
-      <c r="B50" t="s">
-        <v>10</v>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Flash</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C50">
         <v>28500</v>
@@ -2380,12 +1849,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>59</v>
-      </c>
-      <c r="B51" t="s">
-        <v>10</v>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>FLuffy Gangsters</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C51">
         <v>28500</v>
@@ -2409,12 +1878,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>60</v>
-      </c>
-      <c r="B52" t="s">
-        <v>10</v>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>FlyQuest</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C52">
         <v>28500</v>
@@ -2438,12 +1907,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>61</v>
-      </c>
-      <c r="B53" t="s">
-        <v>10</v>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>FlyQuest RED</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C53">
         <v>28500</v>
@@ -2467,12 +1936,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>62</v>
-      </c>
-      <c r="B54" t="s">
-        <v>10</v>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Fnatic</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C54">
         <v>30300</v>
@@ -2496,12 +1965,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>63</v>
-      </c>
-      <c r="B55" t="s">
-        <v>10</v>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>FORZE</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C55">
         <v>28500</v>
@@ -2525,12 +1994,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>64</v>
-      </c>
-      <c r="B56" t="s">
-        <v>10</v>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>FURIA</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C56">
         <v>30300</v>
@@ -2554,12 +2023,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>65</v>
-      </c>
-      <c r="B57" t="s">
-        <v>10</v>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>G2</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C57">
         <v>42100</v>
@@ -2583,12 +2052,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>66</v>
-      </c>
-      <c r="B58" t="s">
-        <v>10</v>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Galorys</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C58">
         <v>28500</v>
@@ -2612,12 +2081,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>67</v>
-      </c>
-      <c r="B59" t="s">
-        <v>10</v>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Gambit</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C59">
         <v>28500</v>
@@ -2641,12 +2110,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>68</v>
-      </c>
-      <c r="B60" t="s">
-        <v>10</v>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>GamerLegion</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C60">
         <v>28500</v>
@@ -2670,12 +2139,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>69</v>
-      </c>
-      <c r="B61" t="s">
-        <v>10</v>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>GATERON</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C61">
         <v>28500</v>
@@ -2699,12 +2168,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>70</v>
-      </c>
-      <c r="B62" t="s">
-        <v>10</v>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>GhoulsW</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C62">
         <v>28500</v>
@@ -2728,12 +2197,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>71</v>
-      </c>
-      <c r="B63" t="s">
-        <v>10</v>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Gods Reign</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C63">
         <v>28500</v>
@@ -2757,12 +2226,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>72</v>
-      </c>
-      <c r="B64" t="s">
-        <v>10</v>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>GODSENT</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C64">
         <v>28500</v>
@@ -2786,12 +2255,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>73</v>
-      </c>
-      <c r="B65" t="s">
-        <v>10</v>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>HAVU</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C65">
         <v>28500</v>
@@ -2815,12 +2284,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>74</v>
-      </c>
-      <c r="B66" t="s">
-        <v>10</v>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Heroic</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C66">
         <v>44900</v>
@@ -2844,12 +2313,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>75</v>
-      </c>
-      <c r="B67" t="s">
-        <v>10</v>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Heroic Academy</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C67">
         <v>28500</v>
@@ -2873,12 +2342,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>76</v>
-      </c>
-      <c r="B68" t="s">
-        <v>10</v>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Hesta</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C68">
         <v>28500</v>
@@ -2902,12 +2371,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>77</v>
-      </c>
-      <c r="B69" t="s">
-        <v>10</v>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Homyno</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C69">
         <v>28500</v>
@@ -2931,12 +2400,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>78</v>
-      </c>
-      <c r="B70" t="s">
-        <v>10</v>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>hoorai</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C70">
         <v>42100</v>
@@ -2960,12 +2429,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>79</v>
-      </c>
-      <c r="B71" t="s">
-        <v>10</v>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>iBUYPOWER</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C71">
         <v>28500</v>
@@ -2989,12 +2458,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>80</v>
-      </c>
-      <c r="B72" t="s">
-        <v>10</v>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>IHC</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C72">
         <v>28500</v>
@@ -3018,12 +2487,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>81</v>
-      </c>
-      <c r="B73" t="s">
-        <v>82</v>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Iluminar</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Tier 2</v>
       </c>
       <c r="C73">
         <v>566500</v>
@@ -3047,12 +2516,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>83</v>
-      </c>
-      <c r="B74" t="s">
-        <v>10</v>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Immortals</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C74">
         <v>28500</v>
@@ -3076,15 +2545,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>84</v>
-      </c>
-      <c r="B75" t="s">
-        <v>10</v>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Imperial</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C75">
-        <v>28500</v>
+        <v>29700</v>
       </c>
       <c r="D75">
         <v>500</v>
@@ -3105,12 +2574,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>85</v>
-      </c>
-      <c r="B76" t="s">
-        <v>10</v>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>inSanitY</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C76">
         <v>28500</v>
@@ -3134,12 +2603,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>86</v>
-      </c>
-      <c r="B77" t="s">
-        <v>10</v>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Into the Beach</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C77">
         <v>28920</v>
@@ -3163,12 +2632,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>87</v>
-      </c>
-      <c r="B78" t="s">
-        <v>10</v>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Kappa Bar</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C78">
         <v>28500</v>
@@ -3192,12 +2661,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>88</v>
-      </c>
-      <c r="B79" t="s">
-        <v>10</v>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>kONO</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C79">
         <v>28500</v>
@@ -3221,12 +2690,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>89</v>
-      </c>
-      <c r="B80" t="s">
-        <v>10</v>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>KRU</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C80">
         <v>28500</v>
@@ -3250,12 +2719,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>90</v>
-      </c>
-      <c r="B81" t="s">
-        <v>10</v>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>LDLC</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C81">
         <v>28500</v>
@@ -3279,12 +2748,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>91</v>
-      </c>
-      <c r="B82" t="s">
-        <v>10</v>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Legacy</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C82">
         <v>28920</v>
@@ -3308,12 +2777,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>92</v>
-      </c>
-      <c r="B83" t="s">
-        <v>10</v>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>LGB</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C83">
         <v>28500</v>
@@ -3337,12 +2806,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>93</v>
-      </c>
-      <c r="B84" t="s">
-        <v>10</v>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Limitless</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C84">
         <v>28500</v>
@@ -3366,12 +2835,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>94</v>
-      </c>
-      <c r="B85" t="s">
-        <v>10</v>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Liquid</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C85">
         <v>97100</v>
@@ -3395,12 +2864,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>95</v>
-      </c>
-      <c r="B86" t="s">
-        <v>10</v>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Luminosity</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C86">
         <v>28500</v>
@@ -3424,15 +2893,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>96</v>
-      </c>
-      <c r="B87" t="s">
-        <v>10</v>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Lynn Vision</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C87">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D87">
         <v>500</v>
@@ -3453,12 +2922,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>97</v>
-      </c>
-      <c r="B88" t="s">
-        <v>10</v>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>M80</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C88">
         <v>28500</v>
@@ -3482,12 +2951,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>98</v>
-      </c>
-      <c r="B89" t="s">
-        <v>10</v>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>MAD Lions</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C89">
         <v>28500</v>
@@ -3511,12 +2980,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>99</v>
-      </c>
-      <c r="B90" t="s">
-        <v>10</v>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>MANA</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C90">
         <v>28500</v>
@@ -3540,12 +3009,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>100</v>
-      </c>
-      <c r="B91" t="s">
-        <v>10</v>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>MenaceGG</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C91">
         <v>28500</v>
@@ -3569,12 +3038,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>101</v>
-      </c>
-      <c r="B92" t="s">
-        <v>10</v>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>MIBR</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C92">
         <v>28500</v>
@@ -3598,12 +3067,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>102</v>
-      </c>
-      <c r="B93" t="s">
-        <v>10</v>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>MIBR Academy</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C93">
         <v>28500</v>
@@ -3627,12 +3096,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>103</v>
-      </c>
-      <c r="B94" t="s">
-        <v>10</v>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Misfits</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C94">
         <v>28500</v>
@@ -3656,12 +3125,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>104</v>
-      </c>
-      <c r="B95" t="s">
-        <v>10</v>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>mousesports</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C95">
         <v>28500</v>
@@ -3685,15 +3154,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>105</v>
-      </c>
-      <c r="B96" t="s">
-        <v>10</v>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>MOUZ</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C96">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D96">
         <v>500</v>
@@ -3714,12 +3183,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>106</v>
-      </c>
-      <c r="B97" t="s">
-        <v>10</v>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>MOUZ NXT</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C97">
         <v>28500</v>
@@ -3743,12 +3212,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>107</v>
-      </c>
-      <c r="B98" t="s">
-        <v>10</v>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Movistar KOI</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C98">
         <v>28500</v>
@@ -3772,12 +3241,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>108</v>
-      </c>
-      <c r="B99" t="s">
-        <v>10</v>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Mythic</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C99">
         <v>28920</v>
@@ -3801,12 +3270,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>109</v>
-      </c>
-      <c r="B100" t="s">
-        <v>10</v>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Natus Vincere</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C100">
         <v>78700</v>
@@ -3830,12 +3299,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>110</v>
-      </c>
-      <c r="B101" t="s">
-        <v>10</v>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>NAVI Junior</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C101">
         <v>42100</v>
@@ -3859,12 +3328,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>111</v>
-      </c>
-      <c r="B102" t="s">
-        <v>10</v>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Nemiga</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C102">
         <v>78700</v>
@@ -3888,12 +3357,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>112</v>
-      </c>
-      <c r="B103" t="s">
-        <v>10</v>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Nexus</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C103">
         <v>28500</v>
@@ -3917,12 +3386,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>113</v>
-      </c>
-      <c r="B104" t="s">
-        <v>10</v>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Ninjas in Pyjamas</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C104">
         <v>28500</v>
@@ -3946,12 +3415,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>114</v>
-      </c>
-      <c r="B105" t="s">
-        <v>10</v>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>NIP Impact</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C105">
         <v>28500</v>
@@ -3975,12 +3444,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>115</v>
-      </c>
-      <c r="B106" t="s">
-        <v>10</v>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>NomadS</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C106">
         <v>28500</v>
@@ -4004,12 +3473,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>116</v>
-      </c>
-      <c r="B107" t="s">
-        <v>10</v>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Nordix</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C107">
         <v>28500</v>
@@ -4033,12 +3502,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>117</v>
-      </c>
-      <c r="B108" t="s">
-        <v>10</v>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>NOVAQ</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C108">
         <v>28500</v>
@@ -4062,12 +3531,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>118</v>
-      </c>
-      <c r="B109" t="s">
-        <v>10</v>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>ODDIK</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C109">
         <v>28500</v>
@@ -4091,12 +3560,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>119</v>
-      </c>
-      <c r="B110" t="s">
-        <v>10</v>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>OG</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C110">
         <v>28500</v>
@@ -4120,12 +3589,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>120</v>
-      </c>
-      <c r="B111" t="s">
-        <v>10</v>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Onyx Ravens</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C111">
         <v>44900</v>
@@ -4149,12 +3618,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>121</v>
-      </c>
-      <c r="B112" t="s">
-        <v>10</v>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Orbit</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C112">
         <v>28500</v>
@@ -4178,12 +3647,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>122</v>
-      </c>
-      <c r="B113" t="s">
-        <v>10</v>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Outsiders</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C113">
         <v>28500</v>
@@ -4207,12 +3676,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>123</v>
-      </c>
-      <c r="B114" t="s">
-        <v>10</v>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>paiN</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C114">
         <v>28500</v>
@@ -4236,12 +3705,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>124</v>
-      </c>
-      <c r="B115" t="s">
-        <v>10</v>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>paiN Academy</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C115">
         <v>28920</v>
@@ -4265,12 +3734,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>125</v>
-      </c>
-      <c r="B116" t="s">
-        <v>10</v>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>PARIVISION</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C116">
         <v>44900</v>
@@ -4294,12 +3763,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>126</v>
-      </c>
-      <c r="B117" t="s">
-        <v>10</v>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Passion UA</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C117">
         <v>28500</v>
@@ -4323,12 +3792,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>127</v>
-      </c>
-      <c r="B118" t="s">
-        <v>10</v>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Permitta</v>
+      </c>
+      <c r="B118" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C118">
         <v>28500</v>
@@ -4352,12 +3821,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>128</v>
-      </c>
-      <c r="B119" t="s">
-        <v>10</v>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Qiang</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C119">
         <v>28500</v>
@@ -4381,12 +3850,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>129</v>
-      </c>
-      <c r="B120" t="s">
-        <v>10</v>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>QMISTRY</v>
+      </c>
+      <c r="B120" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C120">
         <v>28500</v>
@@ -4410,12 +3879,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>130</v>
-      </c>
-      <c r="B121" t="s">
-        <v>10</v>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Quantum Bellator Fire</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C121">
         <v>28500</v>
@@ -4439,12 +3908,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>131</v>
-      </c>
-      <c r="B122" t="s">
-        <v>10</v>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="B122" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C122">
         <v>28500</v>
@@ -4468,12 +3937,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>132</v>
-      </c>
-      <c r="B123" t="s">
-        <v>10</v>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Rebels</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C123">
         <v>42100</v>
@@ -4497,12 +3966,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>133</v>
-      </c>
-      <c r="B124" t="s">
-        <v>10</v>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>RED Canids</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C124">
         <v>28500</v>
@@ -4526,12 +3995,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>134</v>
-      </c>
-      <c r="B125" t="s">
-        <v>10</v>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>Red Viperz</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C125">
         <v>28500</v>
@@ -4555,12 +4024,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>135</v>
-      </c>
-      <c r="B126" t="s">
-        <v>10</v>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>Rogue</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C126">
         <v>28500</v>
@@ -4584,12 +4053,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>136</v>
-      </c>
-      <c r="B127" t="s">
-        <v>10</v>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>Sangal</v>
+      </c>
+      <c r="B127" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C127">
         <v>28500</v>
@@ -4613,12 +4082,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>137</v>
-      </c>
-      <c r="B128" t="s">
-        <v>10</v>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>SAW</v>
+      </c>
+      <c r="B128" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C128">
         <v>28500</v>
@@ -4642,12 +4111,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>138</v>
-      </c>
-      <c r="B129" t="s">
-        <v>10</v>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>Sharks</v>
+      </c>
+      <c r="B129" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C129">
         <v>28500</v>
@@ -4671,12 +4140,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>139</v>
-      </c>
-      <c r="B130" t="s">
-        <v>10</v>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Shika</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C130">
         <v>28500</v>
@@ -4700,12 +4169,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
-        <v>140</v>
-      </c>
-      <c r="B131" t="s">
-        <v>10</v>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>ShindeN</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C131">
         <v>28500</v>
@@ -4729,12 +4198,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>141</v>
-      </c>
-      <c r="B132" t="s">
-        <v>10</v>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>SK</v>
+      </c>
+      <c r="B132" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C132">
         <v>28500</v>
@@ -4758,12 +4227,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>142</v>
-      </c>
-      <c r="B133" t="s">
-        <v>10</v>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>Skinvault</v>
+      </c>
+      <c r="B133" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C133">
         <v>28500</v>
@@ -4787,12 +4256,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>143</v>
-      </c>
-      <c r="B134" t="s">
-        <v>10</v>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>SKYFURY</v>
+      </c>
+      <c r="B134" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C134">
         <v>28920</v>
@@ -4816,12 +4285,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>144</v>
-      </c>
-      <c r="B135" t="s">
-        <v>10</v>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>Space Soldiers</v>
+      </c>
+      <c r="B135" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C135">
         <v>28500</v>
@@ -4845,12 +4314,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>145</v>
-      </c>
-      <c r="B136" t="s">
-        <v>10</v>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>Spirit</v>
+      </c>
+      <c r="B136" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C136">
         <v>44900</v>
@@ -4874,12 +4343,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>146</v>
-      </c>
-      <c r="B137" t="s">
-        <v>10</v>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>Spirit Academy</v>
+      </c>
+      <c r="B137" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C137">
         <v>28500</v>
@@ -4903,12 +4372,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>147</v>
-      </c>
-      <c r="B138" t="s">
-        <v>10</v>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>Sprout</v>
+      </c>
+      <c r="B138" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C138">
         <v>28500</v>
@@ -4932,12 +4401,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>148</v>
-      </c>
-      <c r="B139" t="s">
-        <v>10</v>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>Take Flyte</v>
+      </c>
+      <c r="B139" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C139">
         <v>28920</v>
@@ -4961,12 +4430,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>149</v>
-      </c>
-      <c r="B140" t="s">
-        <v>10</v>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>TALON</v>
+      </c>
+      <c r="B140" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C140">
         <v>42100</v>
@@ -4990,12 +4459,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>150</v>
-      </c>
-      <c r="B141" t="s">
-        <v>10</v>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>Kinguin</v>
+      </c>
+      <c r="B141" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C141">
         <v>28500</v>
@@ -5019,12 +4488,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>151</v>
-      </c>
-      <c r="B142" t="s">
-        <v>10</v>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>Solid</v>
+      </c>
+      <c r="B142" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C142">
         <v>28500</v>
@@ -5048,12 +4517,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>152</v>
-      </c>
-      <c r="B143" t="s">
-        <v>10</v>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>The Dice</v>
+      </c>
+      <c r="B143" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C143">
         <v>28500</v>
@@ -5077,12 +4546,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
-        <v>153</v>
-      </c>
-      <c r="B144" t="s">
-        <v>10</v>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>The Huns</v>
+      </c>
+      <c r="B144" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C144">
         <v>28500</v>
@@ -5106,12 +4575,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
-        <v>154</v>
-      </c>
-      <c r="B145" t="s">
-        <v>82</v>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>The MongolZ</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Tier 2</v>
       </c>
       <c r="C145">
         <v>88700</v>
@@ -5135,12 +4604,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
-        <v>155</v>
-      </c>
-      <c r="B146" t="s">
-        <v>10</v>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>Titan</v>
+      </c>
+      <c r="B146" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C146">
         <v>54500</v>
@@ -5164,12 +4633,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
-        <v>156</v>
-      </c>
-      <c r="B147" t="s">
-        <v>10</v>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>Tricked</v>
+      </c>
+      <c r="B147" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C147">
         <v>28500</v>
@@ -5193,12 +4662,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
-        <v>157</v>
-      </c>
-      <c r="B148" t="s">
-        <v>10</v>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>True Rippers</v>
+      </c>
+      <c r="B148" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C148">
         <v>28500</v>
@@ -5222,12 +4691,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>158</v>
-      </c>
-      <c r="B149" t="s">
-        <v>10</v>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>Tsunami</v>
+      </c>
+      <c r="B149" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C149">
         <v>28500</v>
@@ -5251,12 +4720,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>159</v>
-      </c>
-      <c r="B150" t="s">
-        <v>10</v>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>TYLOO</v>
+      </c>
+      <c r="B150" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C150">
         <v>28500</v>
@@ -5280,12 +4749,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>160</v>
-      </c>
-      <c r="B151" t="s">
-        <v>10</v>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>Underground</v>
+      </c>
+      <c r="B151" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C151">
         <v>28500</v>
@@ -5309,12 +4778,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>161</v>
-      </c>
-      <c r="B152" t="s">
-        <v>10</v>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>Vantage</v>
+      </c>
+      <c r="B152" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C152">
         <v>28500</v>
@@ -5338,12 +4807,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
-        <v>162</v>
-      </c>
-      <c r="B153" t="s">
-        <v>10</v>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>Venom</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C153">
         <v>28500</v>
@@ -5367,12 +4836,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A154" t="s">
-        <v>163</v>
-      </c>
-      <c r="B154" t="s">
-        <v>10</v>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>Verdant</v>
+      </c>
+      <c r="B154" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C154">
         <v>42100</v>
@@ -5396,12 +4865,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A155" t="s">
-        <v>164</v>
-      </c>
-      <c r="B155" t="s">
-        <v>10</v>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>VeryGames</v>
+      </c>
+      <c r="B155" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C155">
         <v>28500</v>
@@ -5425,12 +4894,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A156" t="s">
-        <v>165</v>
-      </c>
-      <c r="B156" t="s">
-        <v>10</v>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>Vexed</v>
+      </c>
+      <c r="B156" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C156">
         <v>28500</v>
@@ -5454,12 +4923,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
-        <v>166</v>
-      </c>
-      <c r="B157" t="s">
-        <v>10</v>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>Victores Sumus</v>
+      </c>
+      <c r="B157" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C157">
         <v>28500</v>
@@ -5483,12 +4952,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
-        <v>167</v>
-      </c>
-      <c r="B158" t="s">
-        <v>10</v>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>Virtus.pro</v>
+      </c>
+      <c r="B158" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C158">
         <v>28500</v>
@@ -5512,15 +4981,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A159" t="s">
-        <v>168</v>
-      </c>
-      <c r="B159" t="s">
-        <v>82</v>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>Vitality</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Tier 2</v>
       </c>
       <c r="C159">
-        <v>196795.23809523811</v>
+        <v>196795.2380952381</v>
       </c>
       <c r="D159">
         <v>500</v>
@@ -5541,12 +5010,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
-        <v>169</v>
-      </c>
-      <c r="B160" t="s">
-        <v>10</v>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>Vox Eminor</v>
+      </c>
+      <c r="B160" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C160">
         <v>29700</v>
@@ -5570,12 +5039,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
-        <v>170</v>
-      </c>
-      <c r="B161" t="s">
-        <v>10</v>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>VP.Prodigy</v>
+      </c>
+      <c r="B161" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C161">
         <v>28500</v>
@@ -5599,12 +5068,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A162" t="s">
-        <v>171</v>
-      </c>
-      <c r="B162" t="s">
-        <v>10</v>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>Wildcard</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C162">
         <v>28500</v>
@@ -5628,12 +5097,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
-        <v>172</v>
-      </c>
-      <c r="B163" t="s">
-        <v>10</v>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>Wildcard Academy</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C163">
         <v>28920</v>
@@ -5657,12 +5126,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
-        <v>173</v>
-      </c>
-      <c r="B164" t="s">
-        <v>10</v>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>Wings Up</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C164">
         <v>28500</v>
@@ -5686,12 +5155,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
-        <v>174</v>
-      </c>
-      <c r="B165" t="s">
-        <v>10</v>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>Wizards</v>
+      </c>
+      <c r="B165" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C165">
         <v>28500</v>
@@ -5715,15 +5184,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
-        <v>175</v>
-      </c>
-      <c r="B166" t="s">
-        <v>10</v>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="B166" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C166">
-        <v>28657</v>
+        <v>30457</v>
       </c>
       <c r="D166">
         <v>500</v>
@@ -5744,12 +5213,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A167" t="s">
-        <v>176</v>
-      </c>
-      <c r="B167" t="s">
-        <v>10</v>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>Core</v>
+      </c>
+      <c r="B167" t="str">
+        <v>Tier 3</v>
       </c>
       <c r="C167">
         <v>0</v>
@@ -5774,9 +5243,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I166" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I167"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>